<commit_message>
Save workspace edits: update agent, app, tools, and logs
</commit_message>
<xml_diff>
--- a/logs/agent_logs.xlsx
+++ b/logs/agent_logs.xlsx
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F78"/>
+  <dimension ref="A1:F91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -3301,6 +3301,464 @@
         </is>
       </c>
     </row>
+    <row r="79">
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>2025-11-13 15:27:26</t>
+        </is>
+      </c>
+      <c r="B79" s="2" t="inlineStr">
+        <is>
+          <t>can you list out all the tables, describe them, get count of rows from all the tables, show all the orders of john, john smith and smith</t>
+        </is>
+      </c>
+      <c r="C79" s="2" t="inlineStr">
+        <is>
+          <t>list_tables, describe_table, describe_table, get_table_row_count, get_table_row_count, nl2sql_query, nl2sql_query, nl2sql_query</t>
+        </is>
+      </c>
+      <c r="D79" s="2" t="inlineStr">
+        <is>
+          <t>No URLs</t>
+        </is>
+      </c>
+      <c r="E79" s="2" t="inlineStr">
+        <is>
+          <t>```markdown
+order_number | product | amount | status | order_date | name
+---|---|---|---|---|---
+ORD-005 | Headphones | 150.0 | Delivered | 2024-11-15 | John Smith
+ORD-006 | Speaker | 200.0 | Shipped | 2024-11-20 | John Smith
+```</t>
+        </is>
+      </c>
+      <c r="F79" s="3" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>2025-11-13 17:19:12</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>list out all the addresses of the students</t>
+        </is>
+      </c>
+      <c r="C80" s="2" t="inlineStr">
+        <is>
+          <t>list_tables, get_table_row_count, describe_table, nl2sql_query</t>
+        </is>
+      </c>
+      <c r="D80" s="2" t="inlineStr">
+        <is>
+          <t>No URLs</t>
+        </is>
+      </c>
+      <c r="E80" s="2" t="inlineStr">
+        <is>
+          <t>It seems that there is no table named 'students' in the database. The available tables are 'customers', 'sqlite_sequence', and 'orders'. Therefore, it is not possible to retrieve the addresses of the students.</t>
+        </is>
+      </c>
+      <c r="F80" s="3" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="inlineStr">
+        <is>
+          <t>2025-11-13 17:27:42</t>
+        </is>
+      </c>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
+          <t>that is not from the database, its from the addresses.csv from RAG</t>
+        </is>
+      </c>
+      <c r="C81" s="2" t="inlineStr">
+        <is>
+          <t>list_tables, get_table_row_count, describe_table, nl2sql_query, nl2sql_query, duckduckgo_results_json</t>
+        </is>
+      </c>
+      <c r="D81" s="2" t="inlineStr">
+        <is>
+          <t>https://pureinsights.com/blog/2024/analyzing-dynamic-tabular-data-in-rag-applications/,
+https://astroa7m.medium.com/converting-csv-files-for-rag-systems-a-concise-guide-856af3d8999a,
+https://towardsdatascience.com/rag-how-to-talk-to-your-data-eaf5469b83b0/
+https://www.machinelearningplus.com/gen-ai/build-a-simple-rag-system-with-csv-files-step-by-step-guide-for-beginners/,</t>
+        </is>
+      </c>
+      <c r="E81" s="2" t="inlineStr">
+        <is>
+          <t>Unfortunately, the available tools and functions do not have the capability to directly retrieve the addresses of the students from the addresses.csv file. However, based on the search results, it appears that there are various approaches to handling dynamic tabular data within RAG systems, including converting CSV files into embeddings for more accurate question answering.
+To retrieve the addresses of the students, you may need to use a different approach, such as loading the CSV file into a database or using a library that supports CSV file processing. Additionally, you may need to modify the RAG system to include the addresses.csv file as a data source.
+If you have any further questions or need help with implementing a solution, please let me know.</t>
+        </is>
+      </c>
+      <c r="F81" s="3" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>2025-11-14 09:40:57</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>can you list out all the addresses from "address_details.csv" , from ./RAG/documents/uploads</t>
+        </is>
+      </c>
+      <c r="C82" s="2" t="inlineStr">
+        <is>
+          <t>list_tables, get_table_row_count, describe_table, nl2sql_query, nl2sql_query, duckduckgo_results_json, visit_web, duckduckgo_results_json, visit_web</t>
+        </is>
+      </c>
+      <c r="D82" s="2" t="inlineStr">
+        <is>
+          <t>https://astroa7m.medium.com/converting-csv-files-for-rag-systems-a-concise-guide-856af3d8999a,
+https://www.addresslabels.app/importing-from-csv-files/:
+https://www.machinelearningplus.com/gen-ai/build-a-simple-rag-system-with-csv-files-step-by-step-guide-for-beginners/,
+https://towardsdatascience.com/rag-how-to-talk-to-your-data-eaf5469b83b0/
+https://www.addresslabels.app/importing-from-csv-files/</t>
+        </is>
+      </c>
+      <c r="E82" s="2" t="inlineStr">
+        <is>
+          <t>Unfortunately, the available tools and functions do not have the capability to directly list out all the addresses from the "address_details.csv" file in the specified directory.
+However, based on the search results, it appears that there are various approaches to handling CSV files, including importing them into a mailing or card list system. One possible solution is to use a library that supports CSV file processing, such as pandas, to read the CSV file and extract the addresses.
+If you have any further questions or need help with implementing a solution, please let me know.</t>
+        </is>
+      </c>
+      <c r="F82" s="3" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="inlineStr">
+        <is>
+          <t>2025-11-14 09:45:32</t>
+        </is>
+      </c>
+      <c r="B83" s="2" t="inlineStr">
+        <is>
+          <t>i am not asking you to write into that file, i am asking to get details from that file</t>
+        </is>
+      </c>
+      <c r="C83" s="2" t="inlineStr">
+        <is>
+          <t>list_tables, get_table_row_count, describe_table, nl2sql_query, nl2sql_query, duckduckgo_results_json, visit_web, duckduckgo_results_json, visit_web, visit_web, duckduckgo_results_json, visit_web, nl2sql_query</t>
+        </is>
+      </c>
+      <c r="D83" s="2" t="inlineStr">
+        <is>
+          <t>https://astroa7m.medium.com/converting-csv-files-for-rag-systems-a-concise-guide-856af3d8999a,
+https://www.addresslabels.app/importing-from-csv-files/:
+https://www.machinelearningplus.com/gen-ai/build-a-simple-rag-system-with-csv-files-step-by-step-guide-for-beginners/,
+https://towardsdatascience.com/rag-how-to-talk-to-your-data-eaf5469b83b0/
+https://www.zhihu.com/question/404356071,</t>
+        </is>
+      </c>
+      <c r="E83" s="2" t="inlineStr">
+        <is>
+          <t>Unfortunately, the available tools and functions do not have the capability to directly read the CSV file "address_details.csv" in the specified directory.
+However, based on the search results, it appears that you can use the pandas library in Python to read a CSV file. The command to read a CSV file using pandas is `pd.read_csv('address_details.csv')`.
+If you have any further questions or need help with implementing a solution, please let me know.</t>
+        </is>
+      </c>
+      <c r="F83" s="3" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>2025-11-14 09:49:51</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
+          <t>use , search_documents tool. or get this data from vector db</t>
+        </is>
+      </c>
+      <c r="C84" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="D84" s="2" t="inlineStr">
+        <is>
+          <t>No URLs</t>
+        </is>
+      </c>
+      <c r="E84" s="2" t="inlineStr">
+        <is>
+          <t>Error: Error code: 400 - {'error': {'message': "tool call validation failed: attempted to call tool 'search_documents' which was not in request.tools", 'type': 'invalid_request_error', 'code': 'tool_use_failed', 'failed_generation': '&lt;function=search_documents&gt;{"query": "address_details.csv in ./RAG/documents/uploads"}&lt;/function&gt;'}}</t>
+        </is>
+      </c>
+      <c r="F84" s="4" t="inlineStr">
+        <is>
+          <t>Error</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="inlineStr">
+        <is>
+          <t>2025-11-14 09:51:17</t>
+        </is>
+      </c>
+      <c r="B85" s="2" t="inlineStr">
+        <is>
+          <t>use rag_tools</t>
+        </is>
+      </c>
+      <c r="C85" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="D85" s="2" t="inlineStr">
+        <is>
+          <t>No URLs</t>
+        </is>
+      </c>
+      <c r="E85" s="2" t="inlineStr">
+        <is>
+          <t>Error: Error code: 400 - {'error': {'message': "tool call validation failed: attempted to call tool 'rag_tools' which was not in request.tools", 'type': 'invalid_request_error', 'code': 'tool_use_failed', 'failed_generation': '&lt;function=rag_tools&gt;{"search_documents": "address_details.csv", "directory": "./RAG/documents/uploads"}"&lt;/function&gt;'}}</t>
+        </is>
+      </c>
+      <c r="F85" s="4" t="inlineStr">
+        <is>
+          <t>Error</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>2025-11-14 11:01:25</t>
+        </is>
+      </c>
+      <c r="B86" s="2" t="inlineStr">
+        <is>
+          <t>list out all the addresses of the students</t>
+        </is>
+      </c>
+      <c r="C86" s="2" t="inlineStr">
+        <is>
+          <t>list_tables, describe_table, nl2sql_query, nl2sql_query</t>
+        </is>
+      </c>
+      <c r="D86" s="2" t="inlineStr">
+        <is>
+          <t>No URLs</t>
+        </is>
+      </c>
+      <c r="E86" s="2" t="inlineStr">
+        <is>
+          <t>Since the database does not have address information or student records, there are no valid results to return for this query. The query results are therefore empty.
+$$
+\boxed{}
+$$</t>
+        </is>
+      </c>
+      <c r="F86" s="3" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="inlineStr">
+        <is>
+          <t>2025-11-14 11:02:17</t>
+        </is>
+      </c>
+      <c r="B87" s="2" t="inlineStr">
+        <is>
+          <t>read address_details.csv</t>
+        </is>
+      </c>
+      <c r="C87" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="D87" s="2" t="inlineStr">
+        <is>
+          <t>No URLs</t>
+        </is>
+      </c>
+      <c r="E87" s="2" t="inlineStr">
+        <is>
+          <t>Error: Error code: 400 - {'error': {'message': "tool call validation failed: attempted to call tool 'read_csv' which was not in request.tools", 'type': 'invalid_request_error', 'code': 'tool_use_failed', 'failed_generation': '&lt;function=read_csv&gt;{"filename": "address_details.csv"}&lt;/function&gt;\n\n'}}</t>
+        </is>
+      </c>
+      <c r="F87" s="4" t="inlineStr">
+        <is>
+          <t>Error</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>2025-11-14 11:06:46</t>
+        </is>
+      </c>
+      <c r="B88" s="2" t="inlineStr">
+        <is>
+          <t>list out all the addresses from the csv</t>
+        </is>
+      </c>
+      <c r="C88" s="2" t="inlineStr">
+        <is>
+          <t>read_csv</t>
+        </is>
+      </c>
+      <c r="D88" s="2" t="inlineStr">
+        <is>
+          <t>No URLs</t>
+        </is>
+      </c>
+      <c r="E88" s="2" t="inlineStr">
+        <is>
+          <t>Here is the list of addresses from the CSV file:
+| street | city | state | zipcode |
+| --- | --- | --- | --- |
+| 12 MG Road | Mumbai | Maharashtra | 400001 |
+| 45 Park Avenue | Ahmedabad | Gujarat | 380015 |
+| 78 Residency Lane | Delhi | Delhi | 110001 |
+| 33 Jubilee Hills | Hyderabad | Telangana | 500033 |
+| 24 Race Course Road | Bengaluru | Karnataka | 560001 |
+| 56 Beach Street | Chennai | Tamil Nadu | 600002 |
+| 19 Green Park | Kochi | Kerala | 682001 |
+| 88 Lake View Road | Pune | Maharashtra | 411001 |
+| 67 Central Avenue | Kolkata | West Bengal | 700001 |
+| 29 Temple Street | Bhopal | Madhya Pradesh | 462001 |
+| 34 Garden Road | Lucknow | Uttar Pradesh | 226001 |
+| 41 Hilltop Street | Jaipur | Rajasthan | 302001 |
+| 53 Riverfront Drive | Surat | Gujarat | 395001 |
+| 62 College Road | Vishakhapatnam | Andhra Pradesh | 530001 |
+| 25 Maple Avenue | Chandigarh | Chandigarh | 160017 |</t>
+        </is>
+      </c>
+      <c r="F88" s="3" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="inlineStr">
+        <is>
+          <t>2025-11-14 11:08:52</t>
+        </is>
+      </c>
+      <c r="B89" s="2" t="inlineStr">
+        <is>
+          <t>Search documents for address</t>
+        </is>
+      </c>
+      <c r="C89" s="2" t="inlineStr">
+        <is>
+          <t>search_documents</t>
+        </is>
+      </c>
+      <c r="D89" s="2" t="inlineStr">
+        <is>
+          <t>No URLs</t>
+        </is>
+      </c>
+      <c r="E89" s="2" t="inlineStr">
+        <is>
+          <t>The search results show 3 relevant documents related to the query "address". The documents are all from the same CSV file, address_details.csv, and contain information about student addresses. The results are listed with their relevance score, source, and content.</t>
+        </is>
+      </c>
+      <c r="F89" s="3" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t>2025-11-14 11:09:53</t>
+        </is>
+      </c>
+      <c r="B90" s="2" t="inlineStr">
+        <is>
+          <t>Search documents for invoice pdf</t>
+        </is>
+      </c>
+      <c r="C90" s="2" t="inlineStr">
+        <is>
+          <t>search_documents, search_documents</t>
+        </is>
+      </c>
+      <c r="D90" s="2" t="inlineStr">
+        <is>
+          <t>No URLs</t>
+        </is>
+      </c>
+      <c r="E90" s="2" t="inlineStr">
+        <is>
+          <t>The search results show 3 relevant documents related to the query "invoice pdf". However, none of the results contain actual invoice PDFs. The results are all from the same Markdown file, agent_self_description.md, and contain information about document chunking and embedding. The relevance score is low, indicating that the results are not very relevant to the query.</t>
+        </is>
+      </c>
+      <c r="F90" s="3" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="inlineStr">
+        <is>
+          <t>2025-11-14 11:11:10</t>
+        </is>
+      </c>
+      <c r="B91" s="2" t="inlineStr">
+        <is>
+          <t>Find in documents address_details.csv</t>
+        </is>
+      </c>
+      <c r="C91" s="2" t="inlineStr">
+        <is>
+          <t>search_documents, search_documents, read_csv</t>
+        </is>
+      </c>
+      <c r="D91" s="2" t="inlineStr">
+        <is>
+          <t>No URLs</t>
+        </is>
+      </c>
+      <c r="E91" s="2" t="inlineStr">
+        <is>
+          <t>The CSV file address_details.csv contains information about addresses. The file has 10 rows and 5 columns: studentnumber, street, city, state, and zipcode. The data includes addresses from various cities in India.</t>
+        </is>
+      </c>
+      <c r="F91" s="3" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>